<commit_message>
Push all latest changes — rasrich_tools app, bank OCR extractor, Schwab fixes, Excel Utilities
- Rename app.py -> stock_processor_page.py; add rasrich_tools.py multi-page entry point
- Add excel_utilities_page.py (Collate Tabs → Master with reconciliation)
- Add _ui_helpers.py, schwab_client_diag.py
- Fix Schwab broker merged Proceeds/Cost layout and update regression baseline
- Add bank statement OCR extractor (claudetestdata CSVs + scripts)
- Add RASRICH Tagger Sprint 1 spec and sample docs
- Update pdf_qc.py, requirements.txt, PARKING_LOT.md, REQUIREMENTS.md, README.md
- Update health baseline: sys_path_hacks 3→4 for schwab_client_diag.py

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testdata/passedtestcases/charles_schwab_drake_import.xlsx
+++ b/testdata/passedtestcases/charles_schwab_drake_import.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="49">
   <si>
     <t>TSJ</t>
   </si>
@@ -143,6 +143,24 @@
   </si>
   <si>
     <t>12/23/2025</t>
+  </si>
+  <si>
+    <t>04/23/2025</t>
+  </si>
+  <si>
+    <t>04/16/2025</t>
+  </si>
+  <si>
+    <t>04/03/2025</t>
+  </si>
+  <si>
+    <t>02/05/2025</t>
+  </si>
+  <si>
+    <t>01/27/2025</t>
+  </si>
+  <si>
+    <t>12/05/2025</t>
   </si>
 </sst>
 </file>
@@ -554,6 +572,9 @@
       <c r="F2" t="s">
         <v>15</v>
       </c>
+      <c r="G2" t="s">
+        <v>29</v>
+      </c>
       <c r="H2" t="s">
         <v>29</v>
       </c>
@@ -568,6 +589,9 @@
       <c r="F3" t="s">
         <v>16</v>
       </c>
+      <c r="G3" t="s">
+        <v>30</v>
+      </c>
       <c r="H3" t="s">
         <v>30</v>
       </c>
@@ -582,6 +606,9 @@
       <c r="F4" t="s">
         <v>17</v>
       </c>
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
       <c r="H4" t="s">
         <v>31</v>
       </c>
@@ -596,8 +623,11 @@
       <c r="F5" t="s">
         <v>18</v>
       </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
       <c r="H5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K5">
         <v>3.44</v>
@@ -610,8 +640,11 @@
       <c r="F6" t="s">
         <v>19</v>
       </c>
+      <c r="G6" t="s">
+        <v>33</v>
+      </c>
       <c r="H6" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="K6">
         <v>389.44</v>
@@ -624,8 +657,11 @@
       <c r="F7" t="s">
         <v>20</v>
       </c>
+      <c r="G7" t="s">
+        <v>34</v>
+      </c>
       <c r="H7" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="K7">
         <v>16.87</v>
@@ -638,8 +674,11 @@
       <c r="F8" t="s">
         <v>21</v>
       </c>
+      <c r="G8" t="s">
+        <v>35</v>
+      </c>
       <c r="H8" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="K8">
         <v>788.85</v>
@@ -652,8 +691,11 @@
       <c r="F9" t="s">
         <v>22</v>
       </c>
+      <c r="G9" t="s">
+        <v>36</v>
+      </c>
       <c r="H9" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="K9">
         <v>1579.4</v>
@@ -666,8 +708,11 @@
       <c r="F10" t="s">
         <v>23</v>
       </c>
+      <c r="G10" t="s">
+        <v>37</v>
+      </c>
       <c r="H10" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="K10">
         <v>44.44</v>
@@ -680,8 +725,11 @@
       <c r="F11" t="s">
         <v>24</v>
       </c>
+      <c r="G11" t="s">
+        <v>38</v>
+      </c>
       <c r="H11" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="K11">
         <v>1618.82</v>
@@ -694,6 +742,9 @@
       <c r="F12" t="s">
         <v>25</v>
       </c>
+      <c r="G12" t="s">
+        <v>39</v>
+      </c>
       <c r="H12" t="s">
         <v>39</v>
       </c>
@@ -708,8 +759,11 @@
       <c r="F13" t="s">
         <v>26</v>
       </c>
+      <c r="G13" t="s">
+        <v>40</v>
+      </c>
       <c r="H13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K13">
         <v>3.44</v>
@@ -722,8 +776,11 @@
       <c r="F14" t="s">
         <v>27</v>
       </c>
+      <c r="G14" t="s">
+        <v>41</v>
+      </c>
       <c r="H14" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="K14">
         <v>174.87</v>
@@ -735,6 +792,9 @@
     <row r="15" spans="1:15">
       <c r="F15" t="s">
         <v>28</v>
+      </c>
+      <c r="G15" t="s">
+        <v>42</v>
       </c>
       <c r="H15" t="s">
         <v>42</v>

</xml_diff>